<commit_message>
modified and ran team_analyzer.py and simulator.py
</commit_message>
<xml_diff>
--- a/output/mariners_report_20260815.xlsx
+++ b/output/mariners_report_20260815.xlsx
@@ -5024,7 +5024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5289,224 +5289,268 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="53" t="inlineStr">
+        <is>
+          <t>WHEN READY</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>ACTIVATE</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>Cooper Criswell (60-day IL)</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>Returning from IL — key contributor</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="53" t="inlineStr">
+        <is>
+          <t>WHEN READY</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>ACTIVATE</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>Matt Brash (15-day IL)</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Returning from IL — key contributor</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>DEADLINE STRATEGY</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="58" t="inlineStr">
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="58" t="inlineStr">
         <is>
           <t>Minor buyer — rotation top 5 MLB, bullpen elite with Brash, offense improving with IL returns. Stand pat or add depth only. Do NOT trade prospects for win-now pieces — system too valuable.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>DEADLINE TARGETS</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="21" t="inlineStr">
-        <is>
-          <t>Position</t>
-        </is>
-      </c>
-      <c r="B19" s="59" t="inlineStr">
-        <is>
-          <t>1B or DH</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="21" t="inlineStr">
-        <is>
-          <t>Profile</t>
-        </is>
-      </c>
-      <c r="B20" s="59" t="inlineStr">
-        <is>
-          <t>Contact/power hybrid — .270+ BA, 20+ HR pace, .340+ xwOBA</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="21" t="inlineStr">
         <is>
-          <t>Cost</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="B21" s="59" t="inlineStr">
         <is>
-          <t>Low-mid prospect or waiver claim</t>
+          <t>1B or DH</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="21" t="inlineStr">
         <is>
-          <t>Urgency</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="B22" s="59" t="inlineStr">
         <is>
-          <t>By July 31</t>
+          <t>Contact/power hybrid — .270+ BA, 20+ HR pace, .340+ xwOBA</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="21" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>Cost</t>
         </is>
       </c>
       <c r="B23" s="59" t="inlineStr">
         <is>
-          <t>1B WAR rank 28-30/30 — Naylor below average bat and glove</t>
+          <t>Low-mid prospect or waiver claim</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>Urgency</t>
+        </is>
+      </c>
+      <c r="B24" s="59" t="inlineStr">
+        <is>
+          <t>By July 31</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="21" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Why</t>
         </is>
       </c>
       <c r="B25" s="59" t="inlineStr">
         <is>
-          <t>RP</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="21" t="inlineStr">
-        <is>
-          <t>Profile</t>
-        </is>
-      </c>
-      <c r="B26" s="59" t="inlineStr">
-        <is>
-          <t>Veteran middle reliever — command-first, groundball tendency</t>
+          <t>1B WAR rank 28-30/30 — Naylor below average bat and glove</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="21" t="inlineStr">
         <is>
-          <t>Cost</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="B27" s="59" t="inlineStr">
         <is>
-          <t>Waiver claim or minimum salary</t>
+          <t>RP</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="21" t="inlineStr">
         <is>
-          <t>Urgency</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="B28" s="59" t="inlineStr">
         <is>
-          <t>Immediate — Hoppe/Wilcox DFA leaves depth hole</t>
+          <t>Veteran middle reliever — command-first, groundball tendency</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="21" t="inlineStr">
         <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="B29" s="59" t="inlineStr">
+        <is>
+          <t>Waiver claim or minimum salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>Urgency</t>
+        </is>
+      </c>
+      <c r="B30" s="59" t="inlineStr">
+        <is>
+          <t>Immediate — Hoppe/Wilcox DFA leaves depth hole</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
           <t>Why</t>
         </is>
       </c>
-      <c r="B29" s="59" t="inlineStr">
+      <c r="B31" s="59" t="inlineStr">
         <is>
           <t>Need reliable 6th/7th inning arm behind Ferrer/Bazardo/Speier</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="12" t="inlineStr">
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>DO NOT TRADE</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="60" t="inlineStr">
-        <is>
-          <t>✗  Julio Rodriguez    — 10yr/$210M franchise player</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="60" t="inlineStr">
-        <is>
-          <t>✗  Bryce Miller       — xwOBA .221 top 3% MLB, ascending</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="60" t="inlineStr">
         <is>
-          <t>✗  Bryan Woo          — xwOBA .272, above average</t>
+          <t>✗  Julio Rodriguez    — 10yr/$210M franchise player</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="60" t="inlineStr">
         <is>
-          <t>✗  Randy Arozarena    — best bat on team when healthy</t>
+          <t>✗  Bryce Miller       — xwOBA .221 top 3% MLB, ascending</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="60" t="inlineStr">
         <is>
-          <t>✗  Matt Brash         — 0.60 ERA, elite closer</t>
+          <t>✗  Bryan Woo          — xwOBA .272, above average</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="60" t="inlineStr">
         <is>
-          <t>✗  Colt Emerson       — 8yr/$95M franchise cornerstone</t>
+          <t>✗  Randy Arozarena    — best bat on team when healthy</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="60" t="inlineStr">
         <is>
-          <t>✗  Cole Young         — 2.4 WAR, emerging star</t>
+          <t>✗  Matt Brash         — 0.60 ERA, elite closer</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="60" t="inlineStr">
         <is>
+          <t>✗  Colt Emerson       — 8yr/$95M franchise cornerstone</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="60" t="inlineStr">
+        <is>
+          <t>✗  Cole Young         — 2.4 WAR, emerging star</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="60" t="inlineStr">
+        <is>
           <t>✗  Logan Gilbert      — 3.29 ERA, 2.1 WAR, ascending</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="61" t="inlineStr">
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="61" t="inlineStr">
         <is>
           <t>SELL CANDIDATES</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="15" t="inlineStr">
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t>Luis Castillo</t>
         </is>
       </c>
-      <c r="B42" s="54" t="inlineStr">
+      <c r="B44" s="54" t="inlineStr">
         <is>
           <t>ERA 5.00+, expensive contract, rotation 6-deep without him  |  Note: Only if ERA continues above 4.50 through July</t>
         </is>
@@ -5514,32 +5558,32 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="A17:D17"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A20:D20"/>
     <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="B44:D44"/>
     <mergeCell ref="B29:D29"/>
     <mergeCell ref="B28:D28"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A40:D40"/>
     <mergeCell ref="A34:D34"/>
     <mergeCell ref="A39:D39"/>
-    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="B24:D24"/>
     <mergeCell ref="A36:D36"/>
-    <mergeCell ref="B20:D20"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B26:D26"/>
     <mergeCell ref="A41:D41"/>
-    <mergeCell ref="A16:D16"/>
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="A37:D37"/>
     <mergeCell ref="A18:D18"/>
+    <mergeCell ref="B31:D31"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A33:D33"/>
-    <mergeCell ref="A32:D32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7558,7 +7602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G108"/>
+  <dimension ref="A1:G111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -7657,13 +7701,13 @@
         </is>
       </c>
       <c r="B5" s="44" t="n">
-        <v>4.01</v>
+        <v>3.93</v>
       </c>
       <c r="C5" s="44" t="n">
-        <v>3.96</v>
+        <v>3.94</v>
       </c>
       <c r="D5" s="18" t="n">
-        <v>0.506</v>
+        <v>0.498</v>
       </c>
       <c r="E5" s="17" t="n">
         <v>26</v>
@@ -7686,13 +7730,13 @@
         </is>
       </c>
       <c r="B6" s="44" t="n">
-        <v>4.11</v>
+        <v>3.95</v>
       </c>
       <c r="C6" s="44" t="n">
         <v>3.94</v>
       </c>
       <c r="D6" s="18" t="n">
-        <v>0.52</v>
+        <v>0.501</v>
       </c>
       <c r="E6" s="17" t="n">
         <v>26</v>
@@ -7715,13 +7759,13 @@
         </is>
       </c>
       <c r="B7" s="44" t="n">
-        <v>4.01</v>
+        <v>3.9</v>
       </c>
       <c r="C7" s="44" t="n">
-        <v>3.99</v>
+        <v>3.98</v>
       </c>
       <c r="D7" s="18" t="n">
-        <v>0.503</v>
+        <v>0.491</v>
       </c>
       <c r="E7" s="17" t="n">
         <v>26</v>
@@ -7744,13 +7788,13 @@
         </is>
       </c>
       <c r="B8" s="44" t="n">
-        <v>4.11</v>
+        <v>3.98</v>
       </c>
       <c r="C8" s="44" t="n">
         <v>3.92</v>
       </c>
       <c r="D8" s="18" t="n">
-        <v>0.521</v>
+        <v>0.507</v>
       </c>
       <c r="E8" s="17" t="n">
         <v>26</v>
@@ -7773,13 +7817,13 @@
         </is>
       </c>
       <c r="B9" s="44" t="n">
-        <v>4.11</v>
+        <v>3.92</v>
       </c>
       <c r="C9" s="44" t="n">
-        <v>3.97</v>
+        <v>3.98</v>
       </c>
       <c r="D9" s="18" t="n">
-        <v>0.516</v>
+        <v>0.493</v>
       </c>
       <c r="E9" s="17" t="n">
         <v>26</v>
@@ -7904,7 +7948,7 @@
         </is>
       </c>
       <c r="B22" s="62" t="n">
-        <v>4.01</v>
+        <v>3.93</v>
       </c>
     </row>
     <row r="23">
@@ -7914,7 +7958,7 @@
         </is>
       </c>
       <c r="B23" s="62" t="n">
-        <v>3.96</v>
+        <v>3.94</v>
       </c>
     </row>
     <row r="24">
@@ -7924,7 +7968,7 @@
         </is>
       </c>
       <c r="B24" s="62" t="n">
-        <v>0.506</v>
+        <v>0.498</v>
       </c>
     </row>
     <row r="25">
@@ -8015,7 +8059,7 @@
       </c>
       <c r="B31" s="34" t="inlineStr">
         <is>
-          <t>+0.040</t>
+          <t>+0.006</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
@@ -8025,7 +8069,7 @@
       </c>
       <c r="D31" s="22" t="inlineStr">
         <is>
-          <t>Bench depth -- status not reconfirmed 2026-08-03, treat this date as stale until verified</t>
+          <t>Bench depth -- confirmed still on 60-day IL (thumb) as of Aug 6-9, no target date reported</t>
         </is>
       </c>
     </row>
@@ -8037,7 +8081,7 @@
       </c>
       <c r="B32" s="34" t="inlineStr">
         <is>
-          <t>+0.100</t>
+          <t>+0.052</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
@@ -8047,14 +8091,14 @@
       </c>
       <c r="D32" s="22" t="inlineStr">
         <is>
-          <t>Elite OBP/walk rate -- 10-day IL, wrist inflammation, placed Jul 19 (Rivas recalled in corresponding move)</t>
+          <t>Elite OBP/walk rate -- still on IL as of Aug 14 (confirmed via live bbref fetch), well past the earlier Aug 2 estimate. Re-verify before trusting this date either.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="21" t="inlineStr">
         <is>
-          <t>IL return: Matt Brash</t>
+          <t>IL return: Cole Wilcox</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
@@ -8064,19 +8108,19 @@
       </c>
       <c r="C33" s="34" t="inlineStr">
         <is>
-          <t>-0.077</t>
+          <t>-0.021</t>
         </is>
       </c>
       <c r="D33" s="22" t="inlineStr">
         <is>
-          <t>0.54 ERA closer -- right lat inflammation, targeting Aug 22-28 return</t>
+          <t>Left oblique strain, placed Aug 7. Was a dependable reliever pre-injury (4.00 ERA, 27 IP) -- no official target date reported yet</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="21" t="inlineStr">
         <is>
-          <t>IL return: Carlos Vargas</t>
+          <t>IL return: Matt Brash</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
@@ -8086,19 +8130,19 @@
       </c>
       <c r="C34" s="34" t="inlineStr">
         <is>
-          <t>-0.050</t>
+          <t>-0.077</t>
         </is>
       </c>
       <c r="D34" s="22" t="inlineStr">
         <is>
-          <t>Bullpen depth -- right lat strain, tentatively scheduled to return Aug 15</t>
+          <t>0.54 ERA closer -- right lat inflammation, targeting Aug 22-28 return</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="21" t="inlineStr">
         <is>
-          <t>IL return: Cooper Criswell</t>
+          <t>IL return: Carlos Vargas</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
@@ -8108,185 +8152,185 @@
       </c>
       <c r="C35" s="34" t="inlineStr">
         <is>
-          <t>-0.026</t>
+          <t>-0.042</t>
         </is>
       </c>
       <c r="D35" s="22" t="inlineStr">
         <is>
-          <t>Right shoulder/pec strain -- targeting Aug 28-Sept 1 return</t>
+          <t>Bullpen depth -- right lat strain, beginning rehab assignment as of mid-Aug after missing 116 straight games</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="21" t="inlineStr">
         <is>
+          <t>IL return: Cooper Criswell</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C36" s="34" t="inlineStr">
+        <is>
+          <t>-0.026</t>
+        </is>
+      </c>
+      <c r="D36" s="22" t="inlineStr">
+        <is>
+          <t>Right shoulder/pec strain -- targeting Aug 28-Sept 1 return</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="21" t="inlineStr">
+        <is>
           <t>Luck correction</t>
         </is>
       </c>
-      <c r="B36" s="8" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C36" s="8" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D36" s="22" t="inlineStr">
+      <c r="D37" s="22" t="inlineStr">
         <is>
           <t>Luck -1.0 - ~0 free wins</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>IL RETURNS + WARD + DOMINGUEZ</t>
         </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="21" t="inlineStr">
-        <is>
-          <t>RS/G</t>
-        </is>
-      </c>
-      <c r="B39" s="62" t="n">
-        <v>4.11</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="21" t="inlineStr">
         <is>
-          <t>RA/G</t>
+          <t>RS/G</t>
         </is>
       </c>
       <c r="B40" s="62" t="n">
-        <v>3.94</v>
+        <v>3.95</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="21" t="inlineStr">
         <is>
-          <t>Win%</t>
+          <t>RA/G</t>
         </is>
       </c>
       <c r="B41" s="62" t="n">
-        <v>0.52</v>
+        <v>3.94</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="21" t="inlineStr">
         <is>
-          <t>Luck wins</t>
+          <t>Win%</t>
         </is>
       </c>
       <c r="B42" s="62" t="n">
-        <v>0</v>
+        <v>0.501</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="21" t="inlineStr">
         <is>
-          <t>Final W-L</t>
-        </is>
-      </c>
-      <c r="B43" s="62" t="inlineStr">
-        <is>
-          <t>83-79</t>
-        </is>
+          <t>Luck wins</t>
+        </is>
+      </c>
+      <c r="B43" s="62" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="21" t="inlineStr">
         <is>
-          <t>Playoff</t>
+          <t>Final W-L</t>
         </is>
       </c>
       <c r="B44" s="62" t="inlineStr">
         <is>
-          <t>Wild Card 3 (bubble)</t>
+          <t>83-79</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="21" t="inlineStr">
         <is>
-          <t>vs TEX</t>
+          <t>Playoff</t>
         </is>
       </c>
       <c r="B45" s="62" t="inlineStr">
         <is>
-          <t>+0 games</t>
+          <t>Wild Card 3 (bubble)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="21" t="inlineStr">
         <is>
+          <t>vs TEX</t>
+        </is>
+      </c>
+      <c r="B46" s="62" t="inlineStr">
+        <is>
+          <t>+0 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="21" t="inlineStr">
+        <is>
           <t>vs HOU</t>
         </is>
       </c>
-      <c r="B46" s="62" t="inlineStr">
+      <c r="B47" s="62" t="inlineStr">
         <is>
           <t>+4 games</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>Factor</t>
         </is>
       </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>RS/G impact</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr">
+      <c r="C48" s="5" t="inlineStr">
         <is>
           <t>RA/G impact</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr">
+      <c r="D48" s="5" t="inlineStr">
         <is>
           <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="21" t="inlineStr">
-        <is>
-          <t>IL return: Will Wilson</t>
-        </is>
-      </c>
-      <c r="B48" s="34" t="inlineStr">
-        <is>
-          <t>+0.040</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D48" s="22" t="inlineStr">
-        <is>
-          <t>Bench depth -- status not reconfirmed 2026-08-03, treat this date as stale until verified</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="21" t="inlineStr">
         <is>
-          <t>IL return: J.P. Crawford</t>
+          <t>IL return: Will Wilson</t>
         </is>
       </c>
       <c r="B49" s="34" t="inlineStr">
         <is>
-          <t>+0.100</t>
+          <t>+0.006</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
@@ -8296,36 +8340,36 @@
       </c>
       <c r="D49" s="22" t="inlineStr">
         <is>
-          <t>Elite OBP/walk rate -- 10-day IL, wrist inflammation, placed Jul 19 (Rivas recalled in corresponding move)</t>
+          <t>Bench depth -- confirmed still on 60-day IL (thumb) as of Aug 6-9, no target date reported</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="21" t="inlineStr">
         <is>
-          <t>IL return: Matt Brash</t>
-        </is>
-      </c>
-      <c r="B50" s="8" t="inlineStr">
+          <t>IL return: J.P. Crawford</t>
+        </is>
+      </c>
+      <c r="B50" s="34" t="inlineStr">
+        <is>
+          <t>+0.052</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C50" s="34" t="inlineStr">
-        <is>
-          <t>-0.077</t>
-        </is>
-      </c>
       <c r="D50" s="22" t="inlineStr">
         <is>
-          <t>0.54 ERA closer -- right lat inflammation, targeting Aug 22-28 return</t>
+          <t>Elite OBP/walk rate -- still on IL as of Aug 14 (confirmed via live bbref fetch), well past the earlier Aug 2 estimate. Re-verify before trusting this date either.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="21" t="inlineStr">
         <is>
-          <t>IL return: Carlos Vargas</t>
+          <t>IL return: Cole Wilcox</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
@@ -8335,19 +8379,19 @@
       </c>
       <c r="C51" s="34" t="inlineStr">
         <is>
-          <t>-0.050</t>
+          <t>-0.021</t>
         </is>
       </c>
       <c r="D51" s="22" t="inlineStr">
         <is>
-          <t>Bullpen depth -- right lat strain, tentatively scheduled to return Aug 15</t>
+          <t>Left oblique strain, placed Aug 7. Was a dependable reliever pre-injury (4.00 ERA, 27 IP) -- no official target date reported yet</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="21" t="inlineStr">
         <is>
-          <t>IL return: Cooper Criswell</t>
+          <t>IL return: Matt Brash</t>
         </is>
       </c>
       <c r="B52" s="8" t="inlineStr">
@@ -8357,41 +8401,41 @@
       </c>
       <c r="C52" s="34" t="inlineStr">
         <is>
-          <t>-0.026</t>
+          <t>-0.077</t>
         </is>
       </c>
       <c r="D52" s="22" t="inlineStr">
         <is>
-          <t>Right shoulder/pec strain -- targeting Aug 28-Sept 1 return</t>
+          <t>0.54 ERA closer -- right lat inflammation, targeting Aug 22-28 return</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="21" t="inlineStr">
         <is>
-          <t>Acquired: Taylor Ward</t>
-        </is>
-      </c>
-      <c r="B53" s="34" t="inlineStr">
-        <is>
-          <t>+0.100</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
+          <t>IL return: Carlos Vargas</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
+      <c r="C53" s="34" t="inlineStr">
+        <is>
+          <t>-0.042</t>
+        </is>
+      </c>
       <c r="D53" s="22" t="inlineStr">
         <is>
-          <t>Acquired from BAL 2026-08-03. .383 OBP -- highest of any regular in the lineup. Pushes Robles to bench.</t>
+          <t>Bullpen depth -- right lat strain, beginning rehab assignment as of mid-Aug after missing 116 straight games</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="21" t="inlineStr">
         <is>
-          <t>Acquired: Seranthony Dominguez</t>
+          <t>IL return: Cooper Criswell</t>
         </is>
       </c>
       <c r="B54" s="8" t="inlineStr">
@@ -8401,224 +8445,224 @@
       </c>
       <c r="C54" s="34" t="inlineStr">
         <is>
-          <t>-0.020</t>
+          <t>-0.026</t>
         </is>
       </c>
       <c r="D54" s="22" t="inlineStr">
         <is>
-          <t>Acquired from CHW 2026-08-03 for Castillo. Lost closer job in late June; projects as setup/middle relief behind Munoz, not closer competition.</t>
+          <t>Right shoulder/pec strain -- targeting Aug 28-Sept 1 return</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="21" t="inlineStr">
         <is>
+          <t>Acquired: Taylor Ward</t>
+        </is>
+      </c>
+      <c r="B55" s="34" t="inlineStr">
+        <is>
+          <t>+0.020</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D55" s="22" t="inlineStr">
+        <is>
+          <t>Acquired from BAL 2026-08-03. Rough Mariners debut so far (8 G, .375 OPS) -- small sample, already reflected in team-wide stats, watch for regression toward his established .729 OPS rate either way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Seranthony Dominguez</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D56" s="22" t="inlineStr">
+        <is>
+          <t>Acquired from CHW 2026-08-03 for Castillo. Rough Mariners debut (5 G, 3.1 IP, 10.80 ERA) -- tiny sample, already reflected in team-wide stats. Was already a modest-at-best add per deadline_trade_comparison.py's stat-by-stat breakdown even before this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="21" t="inlineStr">
+        <is>
           <t>Luck correction</t>
         </is>
       </c>
-      <c r="B55" s="8" t="inlineStr">
+      <c r="B57" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C55" s="8" t="inlineStr">
+      <c r="C57" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D55" s="22" t="inlineStr">
+      <c r="D57" s="22" t="inlineStr">
         <is>
           <t>Luck -1.0 - ~0 free wins</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="2" t="inlineStr">
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>WORST CASE - IL RETURNS SLIP/SETBACK</t>
         </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="21" t="inlineStr">
-        <is>
-          <t>RS/G</t>
-        </is>
-      </c>
-      <c r="B58" s="62" t="n">
-        <v>4.01</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="21" t="inlineStr">
-        <is>
-          <t>RA/G</t>
-        </is>
-      </c>
-      <c r="B59" s="62" t="n">
-        <v>3.99</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="21" t="inlineStr">
         <is>
-          <t>Win%</t>
+          <t>RS/G</t>
         </is>
       </c>
       <c r="B60" s="62" t="n">
-        <v>0.503</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="21" t="inlineStr">
         <is>
-          <t>Luck wins</t>
+          <t>RA/G</t>
         </is>
       </c>
       <c r="B61" s="62" t="n">
-        <v>0</v>
+        <v>3.98</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="21" t="inlineStr">
         <is>
-          <t>Final W-L</t>
-        </is>
-      </c>
-      <c r="B62" s="62" t="inlineStr">
-        <is>
-          <t>83-79</t>
-        </is>
+          <t>Win%</t>
+        </is>
+      </c>
+      <c r="B62" s="62" t="n">
+        <v>0.491</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="21" t="inlineStr">
         <is>
-          <t>Playoff</t>
-        </is>
-      </c>
-      <c r="B63" s="62" t="inlineStr">
-        <is>
-          <t>Wild Card 3 (bubble)</t>
-        </is>
+          <t>Luck wins</t>
+        </is>
+      </c>
+      <c r="B63" s="62" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="21" t="inlineStr">
         <is>
-          <t>vs TEX</t>
+          <t>Final W-L</t>
         </is>
       </c>
       <c r="B64" s="62" t="inlineStr">
         <is>
-          <t>+0 games</t>
+          <t>83-79</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="21" t="inlineStr">
         <is>
-          <t>vs HOU</t>
+          <t>Playoff</t>
         </is>
       </c>
       <c r="B65" s="62" t="inlineStr">
         <is>
-          <t>+4 games</t>
+          <t>Wild Card 3 (bubble)</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="5" t="inlineStr">
-        <is>
-          <t>Factor</t>
-        </is>
-      </c>
-      <c r="B66" s="5" t="inlineStr">
-        <is>
-          <t>RS/G impact</t>
-        </is>
-      </c>
-      <c r="C66" s="5" t="inlineStr">
-        <is>
-          <t>RA/G impact</t>
-        </is>
-      </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t>Note</t>
+      <c r="A66" s="21" t="inlineStr">
+        <is>
+          <t>vs TEX</t>
+        </is>
+      </c>
+      <c r="B66" s="62" t="inlineStr">
+        <is>
+          <t>+0 games</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="21" t="inlineStr">
         <is>
-          <t>IL return: Will Wilson</t>
-        </is>
-      </c>
-      <c r="B67" s="34" t="inlineStr">
-        <is>
-          <t>+0.040</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D67" s="22" t="inlineStr">
-        <is>
-          <t>Bench depth -- status not reconfirmed 2026-08-03, treat this date as stale until verified</t>
+          <t>vs HOU</t>
+        </is>
+      </c>
+      <c r="B67" s="62" t="inlineStr">
+        <is>
+          <t>+4 games</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="21" t="inlineStr">
-        <is>
-          <t>IL return: J.P. Crawford</t>
-        </is>
-      </c>
-      <c r="B68" s="34" t="inlineStr">
-        <is>
-          <t>+0.100</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D68" s="22" t="inlineStr">
-        <is>
-          <t>Elite OBP/walk rate -- 10-day IL, wrist inflammation, placed Jul 19 (Rivas recalled in corresponding move)</t>
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>RS/G impact</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>RA/G impact</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="21" t="inlineStr">
         <is>
-          <t>IL return: Matt Brash</t>
-        </is>
-      </c>
-      <c r="B69" s="8" t="inlineStr">
+          <t>IL return: J.P. Crawford</t>
+        </is>
+      </c>
+      <c r="B69" s="34" t="inlineStr">
+        <is>
+          <t>+0.030</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C69" s="34" t="inlineStr">
-        <is>
-          <t>-0.061</t>
-        </is>
-      </c>
       <c r="D69" s="22" t="inlineStr">
         <is>
-          <t>0.54 ERA closer -- right lat inflammation, targeting Aug 22-28 return</t>
+          <t>Elite OBP/walk rate -- still on IL as of Aug 14 (confirmed via live bbref fetch), well past the earlier Aug 2 estimate. Re-verify before trusting this date either.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="21" t="inlineStr">
         <is>
-          <t>IL return: Carlos Vargas</t>
+          <t>IL return: Cole Wilcox</t>
         </is>
       </c>
       <c r="B70" s="8" t="inlineStr">
@@ -8628,246 +8672,246 @@
       </c>
       <c r="C70" s="34" t="inlineStr">
         <is>
-          <t>-0.042</t>
+          <t>-0.012</t>
         </is>
       </c>
       <c r="D70" s="22" t="inlineStr">
         <is>
-          <t>Bullpen depth -- right lat strain, tentatively scheduled to return Aug 15</t>
+          <t>Left oblique strain, placed Aug 7. Was a dependable reliever pre-injury (4.00 ERA, 27 IP) -- no official target date reported yet</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="21" t="inlineStr">
         <is>
+          <t>IL return: Matt Brash</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C71" s="34" t="inlineStr">
+        <is>
+          <t>-0.061</t>
+        </is>
+      </c>
+      <c r="D71" s="22" t="inlineStr">
+        <is>
+          <t>0.54 ERA closer -- right lat inflammation, targeting Aug 22-28 return</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Carlos Vargas</t>
+        </is>
+      </c>
+      <c r="B72" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C72" s="34" t="inlineStr">
+        <is>
+          <t>-0.035</t>
+        </is>
+      </c>
+      <c r="D72" s="22" t="inlineStr">
+        <is>
+          <t>Bullpen depth -- right lat strain, beginning rehab assignment as of mid-Aug after missing 116 straight games</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="21" t="inlineStr">
+        <is>
           <t>IL return: Cooper Criswell</t>
         </is>
       </c>
-      <c r="B71" s="8" t="inlineStr">
+      <c r="B73" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C71" s="34" t="inlineStr">
+      <c r="C73" s="34" t="inlineStr">
         <is>
           <t>-0.021</t>
         </is>
       </c>
-      <c r="D71" s="22" t="inlineStr">
+      <c r="D73" s="22" t="inlineStr">
         <is>
           <t>Right shoulder/pec strain -- targeting Aug 28-Sept 1 return</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="20" customHeight="1">
-      <c r="A73" s="2" t="inlineStr">
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="2" t="inlineStr">
         <is>
           <t>OPTIMISTIC IL - EVERYONE RETURNS EARLY</t>
         </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="21" t="inlineStr">
-        <is>
-          <t>RS/G</t>
-        </is>
-      </c>
-      <c r="B74" s="62" t="n">
-        <v>4.11</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="21" t="inlineStr">
-        <is>
-          <t>RA/G</t>
-        </is>
-      </c>
-      <c r="B75" s="62" t="n">
-        <v>3.92</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="21" t="inlineStr">
         <is>
-          <t>Win%</t>
+          <t>RS/G</t>
         </is>
       </c>
       <c r="B76" s="62" t="n">
-        <v>0.521</v>
+        <v>3.98</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="21" t="inlineStr">
         <is>
-          <t>Luck wins</t>
+          <t>RA/G</t>
         </is>
       </c>
       <c r="B77" s="62" t="n">
-        <v>0</v>
+        <v>3.92</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="21" t="inlineStr">
         <is>
-          <t>Final W-L</t>
-        </is>
-      </c>
-      <c r="B78" s="62" t="inlineStr">
-        <is>
-          <t>83-79</t>
-        </is>
+          <t>Win%</t>
+        </is>
+      </c>
+      <c r="B78" s="62" t="n">
+        <v>0.507</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="21" t="inlineStr">
         <is>
-          <t>Playoff</t>
-        </is>
-      </c>
-      <c r="B79" s="62" t="inlineStr">
-        <is>
-          <t>Wild Card 3 (bubble)</t>
-        </is>
+          <t>Luck wins</t>
+        </is>
+      </c>
+      <c r="B79" s="62" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="21" t="inlineStr">
         <is>
-          <t>vs TEX</t>
+          <t>Final W-L</t>
         </is>
       </c>
       <c r="B80" s="62" t="inlineStr">
         <is>
-          <t>+0 games</t>
+          <t>83-79</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="21" t="inlineStr">
         <is>
-          <t>vs HOU</t>
+          <t>Playoff</t>
         </is>
       </c>
       <c r="B81" s="62" t="inlineStr">
         <is>
-          <t>+4 games</t>
+          <t>Wild Card 3 (bubble)</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="5" t="inlineStr">
-        <is>
-          <t>Factor</t>
-        </is>
-      </c>
-      <c r="B82" s="5" t="inlineStr">
-        <is>
-          <t>RS/G impact</t>
-        </is>
-      </c>
-      <c r="C82" s="5" t="inlineStr">
-        <is>
-          <t>RA/G impact</t>
-        </is>
-      </c>
-      <c r="D82" s="5" t="inlineStr">
-        <is>
-          <t>Note</t>
+      <c r="A82" s="21" t="inlineStr">
+        <is>
+          <t>vs TEX</t>
+        </is>
+      </c>
+      <c r="B82" s="62" t="inlineStr">
+        <is>
+          <t>+0 games</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="21" t="inlineStr">
         <is>
-          <t>IL return: Will Wilson</t>
-        </is>
-      </c>
-      <c r="B83" s="34" t="inlineStr">
-        <is>
-          <t>+0.040</t>
-        </is>
-      </c>
-      <c r="C83" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D83" s="22" t="inlineStr">
-        <is>
-          <t>Bench depth -- status not reconfirmed 2026-08-03, treat this date as stale until verified</t>
+          <t>vs HOU</t>
+        </is>
+      </c>
+      <c r="B83" s="62" t="inlineStr">
+        <is>
+          <t>+4 games</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="21" t="inlineStr">
-        <is>
-          <t>IL return: J.P. Crawford</t>
-        </is>
-      </c>
-      <c r="B84" s="34" t="inlineStr">
-        <is>
-          <t>+0.100</t>
-        </is>
-      </c>
-      <c r="C84" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D84" s="22" t="inlineStr">
-        <is>
-          <t>Elite OBP/walk rate -- 10-day IL, wrist inflammation, placed Jul 19 (Rivas recalled in corresponding move)</t>
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>RS/G impact</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>RA/G impact</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="21" t="inlineStr">
         <is>
-          <t>IL return: Matt Brash</t>
-        </is>
-      </c>
-      <c r="B85" s="8" t="inlineStr">
+          <t>IL return: Will Wilson</t>
+        </is>
+      </c>
+      <c r="B85" s="34" t="inlineStr">
+        <is>
+          <t>+0.012</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C85" s="34" t="inlineStr">
-        <is>
-          <t>-0.089</t>
-        </is>
-      </c>
       <c r="D85" s="22" t="inlineStr">
         <is>
-          <t>0.54 ERA closer -- right lat inflammation, targeting Aug 22-28 return</t>
+          <t>Bench depth -- confirmed still on 60-day IL (thumb) as of Aug 6-9, no target date reported</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="21" t="inlineStr">
         <is>
-          <t>IL return: Carlos Vargas</t>
-        </is>
-      </c>
-      <c r="B86" s="8" t="inlineStr">
+          <t>IL return: J.P. Crawford</t>
+        </is>
+      </c>
+      <c r="B86" s="34" t="inlineStr">
+        <is>
+          <t>+0.077</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C86" s="34" t="inlineStr">
-        <is>
-          <t>-0.050</t>
-        </is>
-      </c>
       <c r="D86" s="22" t="inlineStr">
         <is>
-          <t>Bullpen depth -- right lat strain, tentatively scheduled to return Aug 15</t>
+          <t>Elite OBP/walk rate -- still on IL as of Aug 14 (confirmed via live bbref fetch), well past the earlier Aug 2 estimate. Re-verify before trusting this date either.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="21" t="inlineStr">
         <is>
-          <t>IL return: Cooper Criswell</t>
+          <t>IL return: Cole Wilcox</t>
         </is>
       </c>
       <c r="B87" s="8" t="inlineStr">
@@ -8877,41 +8921,41 @@
       </c>
       <c r="C87" s="34" t="inlineStr">
         <is>
-          <t>-0.028</t>
+          <t>-0.026</t>
         </is>
       </c>
       <c r="D87" s="22" t="inlineStr">
         <is>
-          <t>Right shoulder/pec strain -- targeting Aug 28-Sept 1 return</t>
+          <t>Left oblique strain, placed Aug 7. Was a dependable reliever pre-injury (4.00 ERA, 27 IP) -- no official target date reported yet</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="21" t="inlineStr">
         <is>
-          <t>Acquired: Taylor Ward</t>
-        </is>
-      </c>
-      <c r="B88" s="34" t="inlineStr">
-        <is>
-          <t>+0.100</t>
-        </is>
-      </c>
-      <c r="C88" s="8" t="inlineStr">
+          <t>IL return: Matt Brash</t>
+        </is>
+      </c>
+      <c r="B88" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
+      <c r="C88" s="34" t="inlineStr">
+        <is>
+          <t>-0.089</t>
+        </is>
+      </c>
       <c r="D88" s="22" t="inlineStr">
         <is>
-          <t>Acquired from BAL 2026-08-03. .383 OBP -- highest of any regular in the lineup. Pushes Robles to bench.</t>
+          <t>0.54 ERA closer -- right lat inflammation, targeting Aug 22-28 return</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="21" t="inlineStr">
         <is>
-          <t>Acquired: Seranthony Dominguez</t>
+          <t>IL return: Carlos Vargas</t>
         </is>
       </c>
       <c r="B89" s="8" t="inlineStr">
@@ -8921,19 +8965,19 @@
       </c>
       <c r="C89" s="34" t="inlineStr">
         <is>
-          <t>-0.020</t>
+          <t>-0.047</t>
         </is>
       </c>
       <c r="D89" s="22" t="inlineStr">
         <is>
-          <t>Acquired from CHW 2026-08-03 for Castillo. Lost closer job in late June; projects as setup/middle relief behind Munoz, not closer competition.</t>
+          <t>Bullpen depth -- right lat strain, beginning rehab assignment as of mid-Aug after missing 116 straight games</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="21" t="inlineStr">
         <is>
-          <t>Luck correction</t>
+          <t>IL return: Cooper Criswell</t>
         </is>
       </c>
       <c r="B90" s="8" t="inlineStr">
@@ -8941,226 +8985,226 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C90" s="8" t="inlineStr">
+      <c r="C90" s="34" t="inlineStr">
+        <is>
+          <t>-0.028</t>
+        </is>
+      </c>
+      <c r="D90" s="22" t="inlineStr">
+        <is>
+          <t>Right shoulder/pec strain -- targeting Aug 28-Sept 1 return</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Taylor Ward</t>
+        </is>
+      </c>
+      <c r="B91" s="34" t="inlineStr">
+        <is>
+          <t>+0.020</t>
+        </is>
+      </c>
+      <c r="C91" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D90" s="22" t="inlineStr">
-        <is>
-          <t>Luck -1.0 - ~0 free wins</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="20" customHeight="1">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>PESSIMISTIC IL - SETBACKS, LATE RETURNS</t>
+      <c r="D91" s="22" t="inlineStr">
+        <is>
+          <t>Acquired from BAL 2026-08-03. Rough Mariners debut so far (8 G, .375 OPS) -- small sample, already reflected in team-wide stats, watch for regression toward his established .729 OPS rate either way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Seranthony Dominguez</t>
+        </is>
+      </c>
+      <c r="B92" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D92" s="22" t="inlineStr">
+        <is>
+          <t>Acquired from CHW 2026-08-03 for Castillo. Rough Mariners debut (5 G, 3.1 IP, 10.80 ERA) -- tiny sample, already reflected in team-wide stats. Was already a modest-at-best add per deadline_trade_comparison.py's stat-by-stat breakdown even before this.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="21" t="inlineStr">
         <is>
-          <t>RS/G</t>
-        </is>
-      </c>
-      <c r="B93" s="62" t="n">
-        <v>4.11</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="21" t="inlineStr">
-        <is>
-          <t>RA/G</t>
-        </is>
-      </c>
-      <c r="B94" s="62" t="n">
-        <v>3.97</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="21" t="inlineStr">
-        <is>
-          <t>Win%</t>
-        </is>
-      </c>
-      <c r="B95" s="62" t="n">
-        <v>0.516</v>
+          <t>Luck correction</t>
+        </is>
+      </c>
+      <c r="B93" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D93" s="22" t="inlineStr">
+        <is>
+          <t>Luck -1.0 - ~0 free wins</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>PESSIMISTIC IL - SETBACKS, LATE RETURNS</t>
+        </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="21" t="inlineStr">
         <is>
-          <t>Luck wins</t>
+          <t>RS/G</t>
         </is>
       </c>
       <c r="B96" s="62" t="n">
-        <v>0</v>
+        <v>3.92</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="21" t="inlineStr">
         <is>
-          <t>Final W-L</t>
-        </is>
-      </c>
-      <c r="B97" s="62" t="inlineStr">
-        <is>
-          <t>83-79</t>
-        </is>
+          <t>RA/G</t>
+        </is>
+      </c>
+      <c r="B97" s="62" t="n">
+        <v>3.98</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="21" t="inlineStr">
         <is>
-          <t>Playoff</t>
-        </is>
-      </c>
-      <c r="B98" s="62" t="inlineStr">
-        <is>
-          <t>Wild Card 3 (bubble)</t>
-        </is>
+          <t>Win%</t>
+        </is>
+      </c>
+      <c r="B98" s="62" t="n">
+        <v>0.493</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="21" t="inlineStr">
         <is>
-          <t>vs TEX</t>
-        </is>
-      </c>
-      <c r="B99" s="62" t="inlineStr">
-        <is>
-          <t>+0 games</t>
-        </is>
+          <t>Luck wins</t>
+        </is>
+      </c>
+      <c r="B99" s="62" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="21" t="inlineStr">
         <is>
-          <t>vs HOU</t>
+          <t>Final W-L</t>
         </is>
       </c>
       <c r="B100" s="62" t="inlineStr">
         <is>
-          <t>+4 games</t>
+          <t>83-79</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="5" t="inlineStr">
-        <is>
-          <t>Factor</t>
-        </is>
-      </c>
-      <c r="B101" s="5" t="inlineStr">
-        <is>
-          <t>RS/G impact</t>
-        </is>
-      </c>
-      <c r="C101" s="5" t="inlineStr">
-        <is>
-          <t>RA/G impact</t>
-        </is>
-      </c>
-      <c r="D101" s="5" t="inlineStr">
-        <is>
-          <t>Note</t>
+      <c r="A101" s="21" t="inlineStr">
+        <is>
+          <t>Playoff</t>
+        </is>
+      </c>
+      <c r="B101" s="62" t="inlineStr">
+        <is>
+          <t>Wild Card 3 (bubble)</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="21" t="inlineStr">
         <is>
-          <t>IL return: Will Wilson</t>
-        </is>
-      </c>
-      <c r="B102" s="34" t="inlineStr">
-        <is>
-          <t>+0.040</t>
-        </is>
-      </c>
-      <c r="C102" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D102" s="22" t="inlineStr">
-        <is>
-          <t>Bench depth -- status not reconfirmed 2026-08-03, treat this date as stale until verified</t>
+          <t>vs TEX</t>
+        </is>
+      </c>
+      <c r="B102" s="62" t="inlineStr">
+        <is>
+          <t>+0 games</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="21" t="inlineStr">
         <is>
-          <t>IL return: J.P. Crawford</t>
-        </is>
-      </c>
-      <c r="B103" s="34" t="inlineStr">
-        <is>
-          <t>+0.100</t>
-        </is>
-      </c>
-      <c r="C103" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D103" s="22" t="inlineStr">
-        <is>
-          <t>Elite OBP/walk rate -- 10-day IL, wrist inflammation, placed Jul 19 (Rivas recalled in corresponding move)</t>
+          <t>vs HOU</t>
+        </is>
+      </c>
+      <c r="B103" s="62" t="inlineStr">
+        <is>
+          <t>+4 games</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="21" t="inlineStr">
-        <is>
-          <t>IL return: Matt Brash</t>
-        </is>
-      </c>
-      <c r="B104" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C104" s="34" t="inlineStr">
-        <is>
-          <t>-0.061</t>
-        </is>
-      </c>
-      <c r="D104" s="22" t="inlineStr">
-        <is>
-          <t>0.54 ERA closer -- right lat inflammation, targeting Aug 22-28 return</t>
+      <c r="A104" s="5" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>RS/G impact</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>RA/G impact</t>
+        </is>
+      </c>
+      <c r="D104" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="21" t="inlineStr">
         <is>
-          <t>IL return: Carlos Vargas</t>
-        </is>
-      </c>
-      <c r="B105" s="8" t="inlineStr">
+          <t>IL return: J.P. Crawford</t>
+        </is>
+      </c>
+      <c r="B105" s="34" t="inlineStr">
+        <is>
+          <t>+0.030</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C105" s="34" t="inlineStr">
-        <is>
-          <t>-0.042</t>
-        </is>
-      </c>
       <c r="D105" s="22" t="inlineStr">
         <is>
-          <t>Bullpen depth -- right lat strain, tentatively scheduled to return Aug 15</t>
+          <t>Elite OBP/walk rate -- still on IL as of Aug 14 (confirmed via live bbref fetch), well past the earlier Aug 2 estimate. Re-verify before trusting this date either.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="21" t="inlineStr">
         <is>
-          <t>IL return: Cooper Criswell</t>
+          <t>IL return: Cole Wilcox</t>
         </is>
       </c>
       <c r="B106" s="8" t="inlineStr">
@@ -9170,117 +9214,183 @@
       </c>
       <c r="C106" s="34" t="inlineStr">
         <is>
-          <t>-0.021</t>
+          <t>-0.012</t>
         </is>
       </c>
       <c r="D106" s="22" t="inlineStr">
         <is>
-          <t>Right shoulder/pec strain -- targeting Aug 28-Sept 1 return</t>
+          <t>Left oblique strain, placed Aug 7. Was a dependable reliever pre-injury (4.00 ERA, 27 IP) -- no official target date reported yet</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="21" t="inlineStr">
         <is>
-          <t>Acquired: Taylor Ward</t>
-        </is>
-      </c>
-      <c r="B107" s="34" t="inlineStr">
-        <is>
-          <t>+0.100</t>
-        </is>
-      </c>
-      <c r="C107" s="8" t="inlineStr">
+          <t>IL return: Matt Brash</t>
+        </is>
+      </c>
+      <c r="B107" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
+      <c r="C107" s="34" t="inlineStr">
+        <is>
+          <t>-0.061</t>
+        </is>
+      </c>
       <c r="D107" s="22" t="inlineStr">
         <is>
-          <t>Acquired from BAL 2026-08-03. .383 OBP -- highest of any regular in the lineup. Pushes Robles to bench.</t>
+          <t>0.54 ERA closer -- right lat inflammation, targeting Aug 22-28 return</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="21" t="inlineStr">
         <is>
+          <t>IL return: Carlos Vargas</t>
+        </is>
+      </c>
+      <c r="B108" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C108" s="34" t="inlineStr">
+        <is>
+          <t>-0.035</t>
+        </is>
+      </c>
+      <c r="D108" s="22" t="inlineStr">
+        <is>
+          <t>Bullpen depth -- right lat strain, beginning rehab assignment as of mid-Aug after missing 116 straight games</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Cooper Criswell</t>
+        </is>
+      </c>
+      <c r="B109" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C109" s="34" t="inlineStr">
+        <is>
+          <t>-0.021</t>
+        </is>
+      </c>
+      <c r="D109" s="22" t="inlineStr">
+        <is>
+          <t>Right shoulder/pec strain -- targeting Aug 28-Sept 1 return</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Taylor Ward</t>
+        </is>
+      </c>
+      <c r="B110" s="34" t="inlineStr">
+        <is>
+          <t>+0.020</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D110" s="22" t="inlineStr">
+        <is>
+          <t>Acquired from BAL 2026-08-03. Rough Mariners debut so far (8 G, .375 OPS) -- small sample, already reflected in team-wide stats, watch for regression toward his established .729 OPS rate either way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="21" t="inlineStr">
+        <is>
           <t>Acquired: Seranthony Dominguez</t>
         </is>
       </c>
-      <c r="B108" s="8" t="inlineStr">
+      <c r="B111" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C108" s="34" t="inlineStr">
-        <is>
-          <t>-0.020</t>
-        </is>
-      </c>
-      <c r="D108" s="22" t="inlineStr">
-        <is>
-          <t>Acquired from CHW 2026-08-03 for Castillo. Lost closer job in late June; projects as setup/middle relief behind Munoz, not closer competition.</t>
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D111" s="22" t="inlineStr">
+        <is>
+          <t>Acquired from CHW 2026-08-03 for Castillo. Rough Mariners debut (5 G, 3.1 IP, 10.80 ERA) -- tiny sample, already reflected in team-wide stats. Was already a modest-at-best add per deadline_trade_comparison.py's stat-by-stat breakdown even before this.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="56">
     <mergeCell ref="B42:G42"/>
+    <mergeCell ref="B101:G101"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B60:G60"/>
+    <mergeCell ref="B67:G67"/>
     <mergeCell ref="B98:G98"/>
     <mergeCell ref="B17:G17"/>
     <mergeCell ref="B23:G23"/>
     <mergeCell ref="B61:G61"/>
-    <mergeCell ref="A38:G38"/>
     <mergeCell ref="B13:G13"/>
     <mergeCell ref="B44:G44"/>
+    <mergeCell ref="B82:G82"/>
     <mergeCell ref="B78:G78"/>
     <mergeCell ref="B29:G29"/>
     <mergeCell ref="B19:G19"/>
+    <mergeCell ref="B103:G103"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B99:G99"/>
-    <mergeCell ref="A92:G92"/>
+    <mergeCell ref="A39:G39"/>
     <mergeCell ref="B65:G65"/>
+    <mergeCell ref="B83:G83"/>
     <mergeCell ref="B40:G40"/>
-    <mergeCell ref="B74:G74"/>
-    <mergeCell ref="A73:G73"/>
+    <mergeCell ref="A59:G59"/>
     <mergeCell ref="A11:G11"/>
     <mergeCell ref="B15:G15"/>
     <mergeCell ref="B64:G64"/>
     <mergeCell ref="B24:G24"/>
     <mergeCell ref="B80:G80"/>
-    <mergeCell ref="B95:G95"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B76:G76"/>
-    <mergeCell ref="B94:G94"/>
     <mergeCell ref="B45:G45"/>
     <mergeCell ref="B63:G63"/>
     <mergeCell ref="B41:G41"/>
     <mergeCell ref="B79:G79"/>
     <mergeCell ref="B26:G26"/>
-    <mergeCell ref="B75:G75"/>
     <mergeCell ref="B97:G97"/>
-    <mergeCell ref="B77:G77"/>
     <mergeCell ref="B62:G62"/>
     <mergeCell ref="B100:G100"/>
     <mergeCell ref="B25:G25"/>
+    <mergeCell ref="A75:G75"/>
+    <mergeCell ref="B47:G47"/>
     <mergeCell ref="B16:G16"/>
     <mergeCell ref="B81:G81"/>
     <mergeCell ref="B46:G46"/>
-    <mergeCell ref="B59:G59"/>
     <mergeCell ref="B22:G22"/>
+    <mergeCell ref="B66:G66"/>
     <mergeCell ref="A21:G21"/>
     <mergeCell ref="B27:G27"/>
-    <mergeCell ref="B93:G93"/>
+    <mergeCell ref="B102:G102"/>
+    <mergeCell ref="A95:G95"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="B43:G43"/>
     <mergeCell ref="B12:G12"/>
     <mergeCell ref="B18:G18"/>
-    <mergeCell ref="B58:G58"/>
-    <mergeCell ref="A57:G57"/>
     <mergeCell ref="B96:G96"/>
-    <mergeCell ref="B39:G39"/>
+    <mergeCell ref="B77:G77"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>